<commit_message>
Release V0.2 archive management upgrades
</commit_message>
<xml_diff>
--- a/deliverables/档案迁移导入模板.xlsx
+++ b/deliverables/档案迁移导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="档案导入" sheetId="1" r:id="Rd8e797e22e0a4c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R778c24bc4c8944de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="档案导入" sheetId="1" r:id="R445dc3263cc04421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R75d922f555d64005"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -605,7 +605,9 @@
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -621,7 +623,13 @@
       <x:c r="D1" s="20" t="str">
         <x:v>份数描述</x:v>
       </x:c>
-      <x:c r="E1" s="21" t="str">
+      <x:c r="E1" s="20" t="str">
+        <x:v>原件库存</x:v>
+      </x:c>
+      <x:c r="F1" s="20" t="str">
+        <x:v>复印件库存</x:v>
+      </x:c>
+      <x:c r="G1" s="21" t="str">
         <x:v>电子文件路径</x:v>
       </x:c>
     </x:row>
@@ -630,705 +638,908 @@
       <x:c r="B2" s="35"/>
       <x:c r="C2" s="35"/>
       <x:c r="D2" s="35"/>
-      <x:c r="E2" s="36"/>
+      <x:c r="E2" s="35"/>
+      <x:c r="F2" s="35"/>
+      <x:c r="G2" s="36"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="34"/>
       <x:c r="B3" s="35"/>
       <x:c r="C3" s="35"/>
       <x:c r="D3" s="35"/>
-      <x:c r="E3" s="36"/>
+      <x:c r="E3" s="35"/>
+      <x:c r="F3" s="35"/>
+      <x:c r="G3" s="36"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="34"/>
       <x:c r="B4" s="35"/>
       <x:c r="C4" s="35"/>
       <x:c r="D4" s="35"/>
-      <x:c r="E4" s="36"/>
+      <x:c r="E4" s="35"/>
+      <x:c r="F4" s="35"/>
+      <x:c r="G4" s="36"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="34"/>
       <x:c r="B5" s="35"/>
       <x:c r="C5" s="35"/>
       <x:c r="D5" s="35"/>
-      <x:c r="E5" s="36"/>
+      <x:c r="E5" s="35"/>
+      <x:c r="F5" s="35"/>
+      <x:c r="G5" s="36"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="34"/>
       <x:c r="B6" s="35"/>
       <x:c r="C6" s="35"/>
       <x:c r="D6" s="35"/>
-      <x:c r="E6" s="36"/>
+      <x:c r="E6" s="35"/>
+      <x:c r="F6" s="35"/>
+      <x:c r="G6" s="36"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="34"/>
       <x:c r="B7" s="35"/>
       <x:c r="C7" s="35"/>
       <x:c r="D7" s="35"/>
-      <x:c r="E7" s="36"/>
+      <x:c r="E7" s="35"/>
+      <x:c r="F7" s="35"/>
+      <x:c r="G7" s="36"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="34"/>
       <x:c r="B8" s="35"/>
       <x:c r="C8" s="35"/>
       <x:c r="D8" s="35"/>
-      <x:c r="E8" s="36"/>
+      <x:c r="E8" s="35"/>
+      <x:c r="F8" s="35"/>
+      <x:c r="G8" s="36"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="34"/>
       <x:c r="B9" s="35"/>
       <x:c r="C9" s="35"/>
       <x:c r="D9" s="35"/>
-      <x:c r="E9" s="36"/>
+      <x:c r="E9" s="35"/>
+      <x:c r="F9" s="35"/>
+      <x:c r="G9" s="36"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="34"/>
       <x:c r="B10" s="35"/>
       <x:c r="C10" s="35"/>
       <x:c r="D10" s="35"/>
-      <x:c r="E10" s="36"/>
+      <x:c r="E10" s="35"/>
+      <x:c r="F10" s="35"/>
+      <x:c r="G10" s="36"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="34"/>
       <x:c r="B11" s="35"/>
       <x:c r="C11" s="35"/>
       <x:c r="D11" s="35"/>
-      <x:c r="E11" s="36"/>
+      <x:c r="E11" s="35"/>
+      <x:c r="F11" s="35"/>
+      <x:c r="G11" s="36"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="34"/>
       <x:c r="B12" s="35"/>
       <x:c r="C12" s="35"/>
       <x:c r="D12" s="35"/>
-      <x:c r="E12" s="36"/>
+      <x:c r="E12" s="35"/>
+      <x:c r="F12" s="35"/>
+      <x:c r="G12" s="36"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="34"/>
       <x:c r="B13" s="35"/>
       <x:c r="C13" s="35"/>
       <x:c r="D13" s="35"/>
-      <x:c r="E13" s="36"/>
+      <x:c r="E13" s="35"/>
+      <x:c r="F13" s="35"/>
+      <x:c r="G13" s="36"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="34"/>
       <x:c r="B14" s="35"/>
       <x:c r="C14" s="35"/>
       <x:c r="D14" s="35"/>
-      <x:c r="E14" s="36"/>
+      <x:c r="E14" s="35"/>
+      <x:c r="F14" s="35"/>
+      <x:c r="G14" s="36"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="34"/>
       <x:c r="B15" s="35"/>
       <x:c r="C15" s="35"/>
       <x:c r="D15" s="35"/>
-      <x:c r="E15" s="36"/>
+      <x:c r="E15" s="35"/>
+      <x:c r="F15" s="35"/>
+      <x:c r="G15" s="36"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="34"/>
       <x:c r="B16" s="35"/>
       <x:c r="C16" s="35"/>
       <x:c r="D16" s="35"/>
-      <x:c r="E16" s="36"/>
+      <x:c r="E16" s="35"/>
+      <x:c r="F16" s="35"/>
+      <x:c r="G16" s="36"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="34"/>
       <x:c r="B17" s="35"/>
       <x:c r="C17" s="35"/>
       <x:c r="D17" s="35"/>
-      <x:c r="E17" s="36"/>
+      <x:c r="E17" s="35"/>
+      <x:c r="F17" s="35"/>
+      <x:c r="G17" s="36"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="34"/>
       <x:c r="B18" s="35"/>
       <x:c r="C18" s="35"/>
       <x:c r="D18" s="35"/>
-      <x:c r="E18" s="36"/>
+      <x:c r="E18" s="35"/>
+      <x:c r="F18" s="35"/>
+      <x:c r="G18" s="36"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="34"/>
       <x:c r="B19" s="35"/>
       <x:c r="C19" s="35"/>
       <x:c r="D19" s="35"/>
-      <x:c r="E19" s="36"/>
+      <x:c r="E19" s="35"/>
+      <x:c r="F19" s="35"/>
+      <x:c r="G19" s="36"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="34"/>
       <x:c r="B20" s="35"/>
       <x:c r="C20" s="35"/>
       <x:c r="D20" s="35"/>
-      <x:c r="E20" s="36"/>
+      <x:c r="E20" s="35"/>
+      <x:c r="F20" s="35"/>
+      <x:c r="G20" s="36"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="34"/>
       <x:c r="B21" s="35"/>
       <x:c r="C21" s="35"/>
       <x:c r="D21" s="35"/>
-      <x:c r="E21" s="36"/>
+      <x:c r="E21" s="35"/>
+      <x:c r="F21" s="35"/>
+      <x:c r="G21" s="36"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="34"/>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
       <x:c r="D22" s="35"/>
-      <x:c r="E22" s="36"/>
+      <x:c r="E22" s="35"/>
+      <x:c r="F22" s="35"/>
+      <x:c r="G22" s="36"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="34"/>
       <x:c r="B23" s="35"/>
       <x:c r="C23" s="35"/>
       <x:c r="D23" s="35"/>
-      <x:c r="E23" s="36"/>
+      <x:c r="E23" s="35"/>
+      <x:c r="F23" s="35"/>
+      <x:c r="G23" s="36"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="34"/>
       <x:c r="B24" s="35"/>
       <x:c r="C24" s="35"/>
       <x:c r="D24" s="35"/>
-      <x:c r="E24" s="36"/>
+      <x:c r="E24" s="35"/>
+      <x:c r="F24" s="35"/>
+      <x:c r="G24" s="36"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="34"/>
       <x:c r="B25" s="35"/>
       <x:c r="C25" s="35"/>
       <x:c r="D25" s="35"/>
-      <x:c r="E25" s="36"/>
+      <x:c r="E25" s="35"/>
+      <x:c r="F25" s="35"/>
+      <x:c r="G25" s="36"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="34"/>
       <x:c r="B26" s="35"/>
       <x:c r="C26" s="35"/>
       <x:c r="D26" s="35"/>
-      <x:c r="E26" s="36"/>
+      <x:c r="E26" s="35"/>
+      <x:c r="F26" s="35"/>
+      <x:c r="G26" s="36"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="34"/>
       <x:c r="B27" s="35"/>
       <x:c r="C27" s="35"/>
       <x:c r="D27" s="35"/>
-      <x:c r="E27" s="36"/>
+      <x:c r="E27" s="35"/>
+      <x:c r="F27" s="35"/>
+      <x:c r="G27" s="36"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="34"/>
       <x:c r="B28" s="35"/>
       <x:c r="C28" s="35"/>
       <x:c r="D28" s="35"/>
-      <x:c r="E28" s="36"/>
+      <x:c r="E28" s="35"/>
+      <x:c r="F28" s="35"/>
+      <x:c r="G28" s="36"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="34"/>
       <x:c r="B29" s="35"/>
       <x:c r="C29" s="35"/>
       <x:c r="D29" s="35"/>
-      <x:c r="E29" s="36"/>
+      <x:c r="E29" s="35"/>
+      <x:c r="F29" s="35"/>
+      <x:c r="G29" s="36"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="34"/>
       <x:c r="B30" s="35"/>
       <x:c r="C30" s="35"/>
       <x:c r="D30" s="35"/>
-      <x:c r="E30" s="36"/>
+      <x:c r="E30" s="35"/>
+      <x:c r="F30" s="35"/>
+      <x:c r="G30" s="36"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="34"/>
       <x:c r="B31" s="35"/>
       <x:c r="C31" s="35"/>
       <x:c r="D31" s="35"/>
-      <x:c r="E31" s="36"/>
+      <x:c r="E31" s="35"/>
+      <x:c r="F31" s="35"/>
+      <x:c r="G31" s="36"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="34"/>
       <x:c r="B32" s="35"/>
       <x:c r="C32" s="35"/>
       <x:c r="D32" s="35"/>
-      <x:c r="E32" s="36"/>
+      <x:c r="E32" s="35"/>
+      <x:c r="F32" s="35"/>
+      <x:c r="G32" s="36"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="34"/>
       <x:c r="B33" s="35"/>
       <x:c r="C33" s="35"/>
       <x:c r="D33" s="35"/>
-      <x:c r="E33" s="36"/>
+      <x:c r="E33" s="35"/>
+      <x:c r="F33" s="35"/>
+      <x:c r="G33" s="36"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="34"/>
       <x:c r="B34" s="35"/>
       <x:c r="C34" s="35"/>
       <x:c r="D34" s="35"/>
-      <x:c r="E34" s="36"/>
+      <x:c r="E34" s="35"/>
+      <x:c r="F34" s="35"/>
+      <x:c r="G34" s="36"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="34"/>
       <x:c r="B35" s="35"/>
       <x:c r="C35" s="35"/>
       <x:c r="D35" s="35"/>
-      <x:c r="E35" s="36"/>
+      <x:c r="E35" s="35"/>
+      <x:c r="F35" s="35"/>
+      <x:c r="G35" s="36"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="34"/>
       <x:c r="B36" s="35"/>
       <x:c r="C36" s="35"/>
       <x:c r="D36" s="35"/>
-      <x:c r="E36" s="36"/>
+      <x:c r="E36" s="35"/>
+      <x:c r="F36" s="35"/>
+      <x:c r="G36" s="36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="34"/>
       <x:c r="B37" s="35"/>
       <x:c r="C37" s="35"/>
       <x:c r="D37" s="35"/>
-      <x:c r="E37" s="36"/>
+      <x:c r="E37" s="35"/>
+      <x:c r="F37" s="35"/>
+      <x:c r="G37" s="36"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="34"/>
       <x:c r="B38" s="35"/>
       <x:c r="C38" s="35"/>
       <x:c r="D38" s="35"/>
-      <x:c r="E38" s="36"/>
+      <x:c r="E38" s="35"/>
+      <x:c r="F38" s="35"/>
+      <x:c r="G38" s="36"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="34"/>
       <x:c r="B39" s="35"/>
       <x:c r="C39" s="35"/>
       <x:c r="D39" s="35"/>
-      <x:c r="E39" s="36"/>
+      <x:c r="E39" s="35"/>
+      <x:c r="F39" s="35"/>
+      <x:c r="G39" s="36"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="34"/>
       <x:c r="B40" s="35"/>
       <x:c r="C40" s="35"/>
       <x:c r="D40" s="35"/>
-      <x:c r="E40" s="36"/>
+      <x:c r="E40" s="35"/>
+      <x:c r="F40" s="35"/>
+      <x:c r="G40" s="36"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="34"/>
       <x:c r="B41" s="35"/>
       <x:c r="C41" s="35"/>
       <x:c r="D41" s="35"/>
-      <x:c r="E41" s="36"/>
+      <x:c r="E41" s="35"/>
+      <x:c r="F41" s="35"/>
+      <x:c r="G41" s="36"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="34"/>
       <x:c r="B42" s="35"/>
       <x:c r="C42" s="35"/>
       <x:c r="D42" s="35"/>
-      <x:c r="E42" s="36"/>
+      <x:c r="E42" s="35"/>
+      <x:c r="F42" s="35"/>
+      <x:c r="G42" s="36"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="34"/>
       <x:c r="B43" s="35"/>
       <x:c r="C43" s="35"/>
       <x:c r="D43" s="35"/>
-      <x:c r="E43" s="36"/>
+      <x:c r="E43" s="35"/>
+      <x:c r="F43" s="35"/>
+      <x:c r="G43" s="36"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="34"/>
       <x:c r="B44" s="35"/>
       <x:c r="C44" s="35"/>
       <x:c r="D44" s="35"/>
-      <x:c r="E44" s="36"/>
+      <x:c r="E44" s="35"/>
+      <x:c r="F44" s="35"/>
+      <x:c r="G44" s="36"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="34"/>
       <x:c r="B45" s="35"/>
       <x:c r="C45" s="35"/>
       <x:c r="D45" s="35"/>
-      <x:c r="E45" s="36"/>
+      <x:c r="E45" s="35"/>
+      <x:c r="F45" s="35"/>
+      <x:c r="G45" s="36"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="34"/>
       <x:c r="B46" s="35"/>
       <x:c r="C46" s="35"/>
       <x:c r="D46" s="35"/>
-      <x:c r="E46" s="36"/>
+      <x:c r="E46" s="35"/>
+      <x:c r="F46" s="35"/>
+      <x:c r="G46" s="36"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="34"/>
       <x:c r="B47" s="35"/>
       <x:c r="C47" s="35"/>
       <x:c r="D47" s="35"/>
-      <x:c r="E47" s="36"/>
+      <x:c r="E47" s="35"/>
+      <x:c r="F47" s="35"/>
+      <x:c r="G47" s="36"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="34"/>
       <x:c r="B48" s="35"/>
       <x:c r="C48" s="35"/>
       <x:c r="D48" s="35"/>
-      <x:c r="E48" s="36"/>
+      <x:c r="E48" s="35"/>
+      <x:c r="F48" s="35"/>
+      <x:c r="G48" s="36"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="34"/>
       <x:c r="B49" s="35"/>
       <x:c r="C49" s="35"/>
       <x:c r="D49" s="35"/>
-      <x:c r="E49" s="36"/>
+      <x:c r="E49" s="35"/>
+      <x:c r="F49" s="35"/>
+      <x:c r="G49" s="36"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="34"/>
       <x:c r="B50" s="35"/>
       <x:c r="C50" s="35"/>
       <x:c r="D50" s="35"/>
-      <x:c r="E50" s="36"/>
+      <x:c r="E50" s="35"/>
+      <x:c r="F50" s="35"/>
+      <x:c r="G50" s="36"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="34"/>
       <x:c r="B51" s="35"/>
       <x:c r="C51" s="35"/>
       <x:c r="D51" s="35"/>
-      <x:c r="E51" s="36"/>
+      <x:c r="E51" s="35"/>
+      <x:c r="F51" s="35"/>
+      <x:c r="G51" s="36"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="34"/>
       <x:c r="B52" s="35"/>
       <x:c r="C52" s="35"/>
       <x:c r="D52" s="35"/>
-      <x:c r="E52" s="36"/>
+      <x:c r="E52" s="35"/>
+      <x:c r="F52" s="35"/>
+      <x:c r="G52" s="36"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="34"/>
       <x:c r="B53" s="35"/>
       <x:c r="C53" s="35"/>
       <x:c r="D53" s="35"/>
-      <x:c r="E53" s="36"/>
+      <x:c r="E53" s="35"/>
+      <x:c r="F53" s="35"/>
+      <x:c r="G53" s="36"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="34"/>
       <x:c r="B54" s="35"/>
       <x:c r="C54" s="35"/>
       <x:c r="D54" s="35"/>
-      <x:c r="E54" s="36"/>
+      <x:c r="E54" s="35"/>
+      <x:c r="F54" s="35"/>
+      <x:c r="G54" s="36"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="34"/>
       <x:c r="B55" s="35"/>
       <x:c r="C55" s="35"/>
       <x:c r="D55" s="35"/>
-      <x:c r="E55" s="36"/>
+      <x:c r="E55" s="35"/>
+      <x:c r="F55" s="35"/>
+      <x:c r="G55" s="36"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="34"/>
       <x:c r="B56" s="35"/>
       <x:c r="C56" s="35"/>
       <x:c r="D56" s="35"/>
-      <x:c r="E56" s="36"/>
+      <x:c r="E56" s="35"/>
+      <x:c r="F56" s="35"/>
+      <x:c r="G56" s="36"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="34"/>
       <x:c r="B57" s="35"/>
       <x:c r="C57" s="35"/>
       <x:c r="D57" s="35"/>
-      <x:c r="E57" s="36"/>
+      <x:c r="E57" s="35"/>
+      <x:c r="F57" s="35"/>
+      <x:c r="G57" s="36"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="34"/>
       <x:c r="B58" s="35"/>
       <x:c r="C58" s="35"/>
       <x:c r="D58" s="35"/>
-      <x:c r="E58" s="36"/>
+      <x:c r="E58" s="35"/>
+      <x:c r="F58" s="35"/>
+      <x:c r="G58" s="36"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="34"/>
       <x:c r="B59" s="35"/>
       <x:c r="C59" s="35"/>
       <x:c r="D59" s="35"/>
-      <x:c r="E59" s="36"/>
+      <x:c r="E59" s="35"/>
+      <x:c r="F59" s="35"/>
+      <x:c r="G59" s="36"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="34"/>
       <x:c r="B60" s="35"/>
       <x:c r="C60" s="35"/>
       <x:c r="D60" s="35"/>
-      <x:c r="E60" s="36"/>
+      <x:c r="E60" s="35"/>
+      <x:c r="F60" s="35"/>
+      <x:c r="G60" s="36"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="34"/>
       <x:c r="B61" s="35"/>
       <x:c r="C61" s="35"/>
       <x:c r="D61" s="35"/>
-      <x:c r="E61" s="36"/>
+      <x:c r="E61" s="35"/>
+      <x:c r="F61" s="35"/>
+      <x:c r="G61" s="36"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="34"/>
       <x:c r="B62" s="35"/>
       <x:c r="C62" s="35"/>
       <x:c r="D62" s="35"/>
-      <x:c r="E62" s="36"/>
+      <x:c r="E62" s="35"/>
+      <x:c r="F62" s="35"/>
+      <x:c r="G62" s="36"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="34"/>
       <x:c r="B63" s="35"/>
       <x:c r="C63" s="35"/>
       <x:c r="D63" s="35"/>
-      <x:c r="E63" s="36"/>
+      <x:c r="E63" s="35"/>
+      <x:c r="F63" s="35"/>
+      <x:c r="G63" s="36"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="34"/>
       <x:c r="B64" s="35"/>
       <x:c r="C64" s="35"/>
       <x:c r="D64" s="35"/>
-      <x:c r="E64" s="36"/>
+      <x:c r="E64" s="35"/>
+      <x:c r="F64" s="35"/>
+      <x:c r="G64" s="36"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="34"/>
       <x:c r="B65" s="35"/>
       <x:c r="C65" s="35"/>
       <x:c r="D65" s="35"/>
-      <x:c r="E65" s="36"/>
+      <x:c r="E65" s="35"/>
+      <x:c r="F65" s="35"/>
+      <x:c r="G65" s="36"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="34"/>
       <x:c r="B66" s="35"/>
       <x:c r="C66" s="35"/>
       <x:c r="D66" s="35"/>
-      <x:c r="E66" s="36"/>
+      <x:c r="E66" s="35"/>
+      <x:c r="F66" s="35"/>
+      <x:c r="G66" s="36"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="34"/>
       <x:c r="B67" s="35"/>
       <x:c r="C67" s="35"/>
       <x:c r="D67" s="35"/>
-      <x:c r="E67" s="36"/>
+      <x:c r="E67" s="35"/>
+      <x:c r="F67" s="35"/>
+      <x:c r="G67" s="36"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="34"/>
       <x:c r="B68" s="35"/>
       <x:c r="C68" s="35"/>
       <x:c r="D68" s="35"/>
-      <x:c r="E68" s="36"/>
+      <x:c r="E68" s="35"/>
+      <x:c r="F68" s="35"/>
+      <x:c r="G68" s="36"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="34"/>
       <x:c r="B69" s="35"/>
       <x:c r="C69" s="35"/>
       <x:c r="D69" s="35"/>
-      <x:c r="E69" s="36"/>
+      <x:c r="E69" s="35"/>
+      <x:c r="F69" s="35"/>
+      <x:c r="G69" s="36"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="34"/>
       <x:c r="B70" s="35"/>
       <x:c r="C70" s="35"/>
       <x:c r="D70" s="35"/>
-      <x:c r="E70" s="36"/>
+      <x:c r="E70" s="35"/>
+      <x:c r="F70" s="35"/>
+      <x:c r="G70" s="36"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="34"/>
       <x:c r="B71" s="35"/>
       <x:c r="C71" s="35"/>
       <x:c r="D71" s="35"/>
-      <x:c r="E71" s="36"/>
+      <x:c r="E71" s="35"/>
+      <x:c r="F71" s="35"/>
+      <x:c r="G71" s="36"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="34"/>
       <x:c r="B72" s="35"/>
       <x:c r="C72" s="35"/>
       <x:c r="D72" s="35"/>
-      <x:c r="E72" s="36"/>
+      <x:c r="E72" s="35"/>
+      <x:c r="F72" s="35"/>
+      <x:c r="G72" s="36"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="34"/>
       <x:c r="B73" s="35"/>
       <x:c r="C73" s="35"/>
       <x:c r="D73" s="35"/>
-      <x:c r="E73" s="36"/>
+      <x:c r="E73" s="35"/>
+      <x:c r="F73" s="35"/>
+      <x:c r="G73" s="36"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="34"/>
       <x:c r="B74" s="35"/>
       <x:c r="C74" s="35"/>
       <x:c r="D74" s="35"/>
-      <x:c r="E74" s="36"/>
+      <x:c r="E74" s="35"/>
+      <x:c r="F74" s="35"/>
+      <x:c r="G74" s="36"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="34"/>
       <x:c r="B75" s="35"/>
       <x:c r="C75" s="35"/>
       <x:c r="D75" s="35"/>
-      <x:c r="E75" s="36"/>
+      <x:c r="E75" s="35"/>
+      <x:c r="F75" s="35"/>
+      <x:c r="G75" s="36"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="34"/>
       <x:c r="B76" s="35"/>
       <x:c r="C76" s="35"/>
       <x:c r="D76" s="35"/>
-      <x:c r="E76" s="36"/>
+      <x:c r="E76" s="35"/>
+      <x:c r="F76" s="35"/>
+      <x:c r="G76" s="36"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="34"/>
       <x:c r="B77" s="35"/>
       <x:c r="C77" s="35"/>
       <x:c r="D77" s="35"/>
-      <x:c r="E77" s="36"/>
+      <x:c r="E77" s="35"/>
+      <x:c r="F77" s="35"/>
+      <x:c r="G77" s="36"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="34"/>
       <x:c r="B78" s="35"/>
       <x:c r="C78" s="35"/>
       <x:c r="D78" s="35"/>
-      <x:c r="E78" s="36"/>
+      <x:c r="E78" s="35"/>
+      <x:c r="F78" s="35"/>
+      <x:c r="G78" s="36"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="34"/>
       <x:c r="B79" s="35"/>
       <x:c r="C79" s="35"/>
       <x:c r="D79" s="35"/>
-      <x:c r="E79" s="36"/>
+      <x:c r="E79" s="35"/>
+      <x:c r="F79" s="35"/>
+      <x:c r="G79" s="36"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="34"/>
       <x:c r="B80" s="35"/>
       <x:c r="C80" s="35"/>
       <x:c r="D80" s="35"/>
-      <x:c r="E80" s="36"/>
+      <x:c r="E80" s="35"/>
+      <x:c r="F80" s="35"/>
+      <x:c r="G80" s="36"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="34"/>
       <x:c r="B81" s="35"/>
       <x:c r="C81" s="35"/>
       <x:c r="D81" s="35"/>
-      <x:c r="E81" s="36"/>
+      <x:c r="E81" s="35"/>
+      <x:c r="F81" s="35"/>
+      <x:c r="G81" s="36"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="34"/>
       <x:c r="B82" s="35"/>
       <x:c r="C82" s="35"/>
       <x:c r="D82" s="35"/>
-      <x:c r="E82" s="36"/>
+      <x:c r="E82" s="35"/>
+      <x:c r="F82" s="35"/>
+      <x:c r="G82" s="36"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="34"/>
       <x:c r="B83" s="35"/>
       <x:c r="C83" s="35"/>
       <x:c r="D83" s="35"/>
-      <x:c r="E83" s="36"/>
+      <x:c r="E83" s="35"/>
+      <x:c r="F83" s="35"/>
+      <x:c r="G83" s="36"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="34"/>
       <x:c r="B84" s="35"/>
       <x:c r="C84" s="35"/>
       <x:c r="D84" s="35"/>
-      <x:c r="E84" s="36"/>
+      <x:c r="E84" s="35"/>
+      <x:c r="F84" s="35"/>
+      <x:c r="G84" s="36"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="34"/>
       <x:c r="B85" s="35"/>
       <x:c r="C85" s="35"/>
       <x:c r="D85" s="35"/>
-      <x:c r="E85" s="36"/>
+      <x:c r="E85" s="35"/>
+      <x:c r="F85" s="35"/>
+      <x:c r="G85" s="36"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="34"/>
       <x:c r="B86" s="35"/>
       <x:c r="C86" s="35"/>
       <x:c r="D86" s="35"/>
-      <x:c r="E86" s="36"/>
+      <x:c r="E86" s="35"/>
+      <x:c r="F86" s="35"/>
+      <x:c r="G86" s="36"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="34"/>
       <x:c r="B87" s="35"/>
       <x:c r="C87" s="35"/>
       <x:c r="D87" s="35"/>
-      <x:c r="E87" s="36"/>
+      <x:c r="E87" s="35"/>
+      <x:c r="F87" s="35"/>
+      <x:c r="G87" s="36"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="34"/>
       <x:c r="B88" s="35"/>
       <x:c r="C88" s="35"/>
       <x:c r="D88" s="35"/>
-      <x:c r="E88" s="36"/>
+      <x:c r="E88" s="35"/>
+      <x:c r="F88" s="35"/>
+      <x:c r="G88" s="36"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="34"/>
       <x:c r="B89" s="35"/>
       <x:c r="C89" s="35"/>
       <x:c r="D89" s="35"/>
-      <x:c r="E89" s="36"/>
+      <x:c r="E89" s="35"/>
+      <x:c r="F89" s="35"/>
+      <x:c r="G89" s="36"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="34"/>
       <x:c r="B90" s="35"/>
       <x:c r="C90" s="35"/>
       <x:c r="D90" s="35"/>
-      <x:c r="E90" s="36"/>
+      <x:c r="E90" s="35"/>
+      <x:c r="F90" s="35"/>
+      <x:c r="G90" s="36"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="34"/>
       <x:c r="B91" s="35"/>
       <x:c r="C91" s="35"/>
       <x:c r="D91" s="35"/>
-      <x:c r="E91" s="36"/>
+      <x:c r="E91" s="35"/>
+      <x:c r="F91" s="35"/>
+      <x:c r="G91" s="36"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="34"/>
       <x:c r="B92" s="35"/>
       <x:c r="C92" s="35"/>
       <x:c r="D92" s="35"/>
-      <x:c r="E92" s="36"/>
+      <x:c r="E92" s="35"/>
+      <x:c r="F92" s="35"/>
+      <x:c r="G92" s="36"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="34"/>
       <x:c r="B93" s="35"/>
       <x:c r="C93" s="35"/>
       <x:c r="D93" s="35"/>
-      <x:c r="E93" s="36"/>
+      <x:c r="E93" s="35"/>
+      <x:c r="F93" s="35"/>
+      <x:c r="G93" s="36"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="34"/>
       <x:c r="B94" s="35"/>
       <x:c r="C94" s="35"/>
       <x:c r="D94" s="35"/>
-      <x:c r="E94" s="36"/>
+      <x:c r="E94" s="35"/>
+      <x:c r="F94" s="35"/>
+      <x:c r="G94" s="36"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="34"/>
       <x:c r="B95" s="35"/>
       <x:c r="C95" s="35"/>
       <x:c r="D95" s="35"/>
-      <x:c r="E95" s="36"/>
+      <x:c r="E95" s="35"/>
+      <x:c r="F95" s="35"/>
+      <x:c r="G95" s="36"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="34"/>
       <x:c r="B96" s="35"/>
       <x:c r="C96" s="35"/>
       <x:c r="D96" s="35"/>
-      <x:c r="E96" s="36"/>
+      <x:c r="E96" s="35"/>
+      <x:c r="F96" s="35"/>
+      <x:c r="G96" s="36"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="34"/>
       <x:c r="B97" s="35"/>
       <x:c r="C97" s="35"/>
       <x:c r="D97" s="35"/>
-      <x:c r="E97" s="36"/>
+      <x:c r="E97" s="35"/>
+      <x:c r="F97" s="35"/>
+      <x:c r="G97" s="36"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="34"/>
       <x:c r="B98" s="35"/>
       <x:c r="C98" s="35"/>
       <x:c r="D98" s="35"/>
-      <x:c r="E98" s="36"/>
+      <x:c r="E98" s="35"/>
+      <x:c r="F98" s="35"/>
+      <x:c r="G98" s="36"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="34"/>
       <x:c r="B99" s="35"/>
       <x:c r="C99" s="35"/>
       <x:c r="D99" s="35"/>
-      <x:c r="E99" s="36"/>
+      <x:c r="E99" s="35"/>
+      <x:c r="F99" s="35"/>
+      <x:c r="G99" s="36"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="34"/>
       <x:c r="B100" s="35"/>
       <x:c r="C100" s="35"/>
       <x:c r="D100" s="35"/>
-      <x:c r="E100" s="36"/>
+      <x:c r="E100" s="35"/>
+      <x:c r="F100" s="35"/>
+      <x:c r="G100" s="36"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="37"/>
       <x:c r="B101" s="38"/>
       <x:c r="C101" s="38"/>
       <x:c r="D101" s="38"/>
-      <x:c r="E101" s="39"/>
+      <x:c r="E101" s="38"/>
+      <x:c r="F101" s="38"/>
+      <x:c r="G101" s="39"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C2:C101">
       <x:formula1>"原件,复印件,电子件,其他"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="E2:F101">
+      <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1398,18 +1609,34 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="53" t="str">
+      <x:c r="A9" s="51" t="str">
+        <x:v>原件库存</x:v>
+      </x:c>
+      <x:c r="B9" s="55" t="str">
+        <x:v>非负整数；不填写时默认按 1 份原件导入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="51" t="str">
+        <x:v>复印件库存</x:v>
+      </x:c>
+      <x:c r="B10" s="55" t="str">
+        <x:v>非负整数；不填写时默认按 0 份复印件导入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="53" t="str">
         <x:v>电子文件路径</x:v>
       </x:c>
-      <x:c r="B9" s="56" t="str">
+      <x:c r="B11" s="56" t="str">
         <x:v>填写 Windows 绝对路径；系统只保存路径，不复制文件。</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="38" customHeight="1">
-      <x:c r="A11" s="59" t="str">
+    <x:row r="13" ht="68" customHeight="1">
+      <x:c r="A13" s="59" t="str">
         <x:v>重要提示</x:v>
       </x:c>
-      <x:c r="B11" s="59" t="str">
+      <x:c r="B13" s="59" t="str">
         <x:v>不要修改“档案导入”工作表的表头，不要增加标题行或合并数据单元格；重复导入会产生重复档案。</x:v>
       </x:c>
     </x:row>

</xml_diff>